<commit_message>
update results excel file
</commit_message>
<xml_diff>
--- a/Results/OSO_results.xlsx
+++ b/Results/OSO_results.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dungnguyen\Dropbox\PTIT-research\anh Phuong\12_MasterThesis (todo-paper1-IJIETAP)\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dungnguyen\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{049EB1BF-87E4-41EB-9391-225FA4B42D9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{796F31AA-7F80-4E78-AA88-7D671DFCF2A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General and Special" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="17">
   <si>
     <t>Parameters</t>
   </si>
@@ -32,10 +32,13 @@
     <t>Greedy</t>
   </si>
   <si>
+    <t>SA</t>
+  </si>
+  <si>
     <t>GA</t>
   </si>
   <si>
-    <t>SA</t>
+    <t>Comparison vs. Greedy</t>
   </si>
   <si>
     <t>p</t>
@@ -61,6 +64,15 @@
   <si>
     <t>Time (s)</t>
   </si>
+  <si>
+    <t>Equal</t>
+  </si>
+  <si>
+    <t>Better</t>
+  </si>
+  <si>
+    <t>Worse</t>
+  </si>
 </sst>
 </file>
 
@@ -70,7 +82,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -88,8 +100,19 @@
       <sz val="9"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -131,8 +154,33 @@
         <fgColor rgb="FFF8F9FA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E4057"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4A6FA5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD4EDDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8D7DA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -155,11 +203,50 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -203,7 +290,24 @@
     <xf numFmtId="164" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -509,7 +613,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N116"/>
+  <dimension ref="A1:P116"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="6" customWidth="1"/>
@@ -522,80 +626,91 @@
     <col min="11" max="11" width="12" customWidth="1"/>
     <col min="12" max="12" width="10" customWidth="1"/>
     <col min="13" max="13" width="12" customWidth="1"/>
-    <col min="14" max="14" width="10" customWidth="1"/>
+    <col min="14" max="15" width="10" customWidth="1"/>
+    <col min="16" max="16" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="16"/>
-      <c r="I1" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="J1" s="16"/>
-      <c r="K1" s="15" t="s">
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="20"/>
+      <c r="I1" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="J1" s="20"/>
+      <c r="K1" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="L1" s="20"/>
+      <c r="M1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="L1" s="16"/>
-      <c r="M1" s="15" t="s">
+      <c r="N1" s="20"/>
+      <c r="O1" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="P1" s="23"/>
+    </row>
+    <row r="2" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="O2" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="N1" s="16"/>
-    </row>
-    <row r="2" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P2" s="15" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>10</v>
       </c>
@@ -638,8 +753,14 @@
       <c r="N3" s="10">
         <v>0.82</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O3" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P3" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="13">
         <v>10</v>
       </c>
@@ -682,8 +803,14 @@
       <c r="N4" s="10">
         <v>0.86299999999999999</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O4" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P4" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>10</v>
       </c>
@@ -726,8 +853,14 @@
       <c r="N5" s="10">
         <v>0.93100000000000005</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O5" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P5" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="13">
         <v>10</v>
       </c>
@@ -770,8 +903,14 @@
       <c r="N6" s="10">
         <v>2.9009999999999998</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O6" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P6" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>10</v>
       </c>
@@ -814,8 +953,14 @@
       <c r="N7" s="10">
         <v>1.1850000000000001</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O7" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P7" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="13">
         <v>10</v>
       </c>
@@ -858,8 +1003,14 @@
       <c r="N8" s="10">
         <v>1.1120000000000001</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O8" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P8" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>10</v>
       </c>
@@ -902,8 +1053,14 @@
       <c r="N9" s="10">
         <v>1.294</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O9" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P9" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="13">
         <v>10</v>
       </c>
@@ -946,8 +1103,14 @@
       <c r="N10" s="10">
         <v>2.5099999999999998</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O10" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P10" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -990,8 +1153,14 @@
       <c r="N11" s="10">
         <v>1.407</v>
       </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O11" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P11" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="13">
         <v>10</v>
       </c>
@@ -1034,8 +1203,14 @@
       <c r="N12" s="10">
         <v>2.7240000000000002</v>
       </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O12" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P12" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>10</v>
       </c>
@@ -1078,8 +1253,14 @@
       <c r="N13" s="10">
         <v>1.5820000000000001</v>
       </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O13" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P13" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="13">
         <v>10</v>
       </c>
@@ -1122,8 +1303,14 @@
       <c r="N14" s="10">
         <v>1.6060000000000001</v>
       </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O14" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P14" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>10</v>
       </c>
@@ -1166,8 +1353,14 @@
       <c r="N15" s="10">
         <v>3.9180000000000001</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O15" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P15" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="13">
         <v>10</v>
       </c>
@@ -1210,8 +1403,14 @@
       <c r="N16" s="10">
         <v>2.2480000000000002</v>
       </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O16" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P16" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>10</v>
       </c>
@@ -1254,8 +1453,14 @@
       <c r="N17" s="10">
         <v>2.2229999999999999</v>
       </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O17" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P17" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="13">
         <v>10</v>
       </c>
@@ -1298,8 +1503,14 @@
       <c r="N18" s="10">
         <v>1.754</v>
       </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O18" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P18" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>10</v>
       </c>
@@ -1342,8 +1553,14 @@
       <c r="N19" s="10">
         <v>1.8480000000000001</v>
       </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O19" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P19" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="13">
         <v>10</v>
       </c>
@@ -1386,8 +1603,14 @@
       <c r="N20" s="10">
         <v>2.532</v>
       </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O20" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P20" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>25</v>
       </c>
@@ -1430,8 +1653,14 @@
       <c r="N21" s="10">
         <v>2.8450000000000002</v>
       </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O21" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P21" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="13">
         <v>25</v>
       </c>
@@ -1474,8 +1703,14 @@
       <c r="N22" s="10">
         <v>2.3050000000000002</v>
       </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O22" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P22" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>25</v>
       </c>
@@ -1518,8 +1753,14 @@
       <c r="N23" s="10">
         <v>0.629</v>
       </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O23" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P23" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="13">
         <v>25</v>
       </c>
@@ -1562,8 +1803,14 @@
       <c r="N24" s="10">
         <v>1.8660000000000001</v>
       </c>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O24" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P24" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>25</v>
       </c>
@@ -1606,8 +1853,14 @@
       <c r="N25" s="10">
         <v>8.5169999999999995</v>
       </c>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O25" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P25" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="13">
         <v>25</v>
       </c>
@@ -1650,8 +1903,14 @@
       <c r="N26" s="10">
         <v>7.8250000000000002</v>
       </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O26" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P26" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>25</v>
       </c>
@@ -1694,8 +1953,14 @@
       <c r="N27" s="10">
         <v>4.0529999999999999</v>
       </c>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O27" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P27" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="13">
         <v>25</v>
       </c>
@@ -1738,8 +2003,14 @@
       <c r="N28" s="10">
         <v>1.3560000000000001</v>
       </c>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O28" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P28" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>25</v>
       </c>
@@ -1782,8 +2053,14 @@
       <c r="N29" s="10">
         <v>4.2809999999999997</v>
       </c>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O29" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P29" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="13">
         <v>25</v>
       </c>
@@ -1826,8 +2103,14 @@
       <c r="N30" s="10">
         <v>4.6529999999999996</v>
       </c>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O30" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P30" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>25</v>
       </c>
@@ -1870,8 +2153,14 @@
       <c r="N31" s="10">
         <v>5.944</v>
       </c>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O31" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P31" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="13">
         <v>25</v>
       </c>
@@ -1914,8 +2203,14 @@
       <c r="N32" s="10">
         <v>1.837</v>
       </c>
-    </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O32" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P32" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>25</v>
       </c>
@@ -1958,8 +2253,14 @@
       <c r="N33" s="10">
         <v>10.507</v>
       </c>
-    </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O33" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P33" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" s="13">
         <v>25</v>
       </c>
@@ -2002,8 +2303,14 @@
       <c r="N34" s="10">
         <v>3.677</v>
       </c>
-    </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O34" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P34" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>25</v>
       </c>
@@ -2046,8 +2353,14 @@
       <c r="N35" s="10">
         <v>6.0990000000000002</v>
       </c>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O35" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P35" s="18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="13">
         <v>25</v>
       </c>
@@ -2090,8 +2403,14 @@
       <c r="N36" s="10">
         <v>3.28</v>
       </c>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O36" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P36" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>25</v>
       </c>
@@ -2134,8 +2453,14 @@
       <c r="N37" s="10">
         <v>17.677</v>
       </c>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O37" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P37" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" s="13">
         <v>25</v>
       </c>
@@ -2178,8 +2503,14 @@
       <c r="N38" s="10">
         <v>9.8529999999999998</v>
       </c>
-    </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O38" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P38" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>25</v>
       </c>
@@ -2222,8 +2553,14 @@
       <c r="N39" s="10">
         <v>8.202</v>
       </c>
-    </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O39" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P39" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="13">
         <v>25</v>
       </c>
@@ -2266,8 +2603,14 @@
       <c r="N40" s="10">
         <v>6.5430000000000001</v>
       </c>
-    </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O40" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P40" s="18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>25</v>
       </c>
@@ -2310,8 +2653,14 @@
       <c r="N41" s="10">
         <v>11.955</v>
       </c>
-    </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O41" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P41" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" s="13">
         <v>25</v>
       </c>
@@ -2354,8 +2703,14 @@
       <c r="N42" s="10">
         <v>15.331</v>
       </c>
-    </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O42" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P42" s="18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>25</v>
       </c>
@@ -2398,8 +2753,14 @@
       <c r="N43" s="10">
         <v>16.381</v>
       </c>
-    </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O43" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P43" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" s="13">
         <v>25</v>
       </c>
@@ -2442,8 +2803,14 @@
       <c r="N44" s="10">
         <v>5.2350000000000003</v>
       </c>
-    </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O44" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P44" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>25</v>
       </c>
@@ -2486,8 +2853,14 @@
       <c r="N45" s="10">
         <v>18.649000000000001</v>
       </c>
-    </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O45" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P45" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="13">
         <v>25</v>
       </c>
@@ -2530,8 +2903,14 @@
       <c r="N46" s="10">
         <v>17.309999999999999</v>
       </c>
-    </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O46" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P46" s="18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>25</v>
       </c>
@@ -2574,8 +2953,14 @@
       <c r="N47" s="10">
         <v>33.677999999999997</v>
       </c>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O47" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P47" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" s="13">
         <v>25</v>
       </c>
@@ -2618,8 +3003,14 @@
       <c r="N48" s="10">
         <v>23.599</v>
       </c>
-    </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O48" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P48" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>30</v>
       </c>
@@ -2662,8 +3053,14 @@
       <c r="N49" s="10">
         <v>4.1509999999999998</v>
       </c>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O49" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P49" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="13">
         <v>30</v>
       </c>
@@ -2706,8 +3103,14 @@
       <c r="N50" s="10">
         <v>4.9080000000000004</v>
       </c>
-    </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O50" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P50" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <v>30</v>
       </c>
@@ -2750,8 +3153,14 @@
       <c r="N51" s="10">
         <v>0.755</v>
       </c>
-    </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O51" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P51" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" s="13">
         <v>30</v>
       </c>
@@ -2794,8 +3203,14 @@
       <c r="N52" s="10">
         <v>0.82599999999999996</v>
       </c>
-    </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O52" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P52" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>30</v>
       </c>
@@ -2838,8 +3253,14 @@
       <c r="N53" s="10">
         <v>6.806</v>
       </c>
-    </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O53" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P53" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="13">
         <v>30</v>
       </c>
@@ -2882,8 +3303,14 @@
       <c r="N54" s="10">
         <v>5.4889999999999999</v>
       </c>
-    </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O54" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P54" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>30</v>
       </c>
@@ -2926,8 +3353,14 @@
       <c r="N55" s="10">
         <v>5.5590000000000002</v>
       </c>
-    </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O55" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P55" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" s="13">
         <v>30</v>
       </c>
@@ -2970,8 +3403,14 @@
       <c r="N56" s="10">
         <v>4.6029999999999998</v>
       </c>
-    </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O56" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P56" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>30</v>
       </c>
@@ -3014,8 +3453,14 @@
       <c r="N57" s="10">
         <v>6.5019999999999998</v>
       </c>
-    </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O57" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="P57" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" s="13">
         <v>30</v>
       </c>
@@ -3058,8 +3503,14 @@
       <c r="N58" s="10">
         <v>3.18</v>
       </c>
-    </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O58" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P58" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>30</v>
       </c>
@@ -3102,8 +3553,14 @@
       <c r="N59" s="10">
         <v>4.4989999999999997</v>
       </c>
-    </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O59" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P59" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" s="13">
         <v>30</v>
       </c>
@@ -3146,8 +3603,14 @@
       <c r="N60" s="10">
         <v>2.3839999999999999</v>
       </c>
-    </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O60" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P60" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>30</v>
       </c>
@@ -3190,8 +3653,14 @@
       <c r="N61" s="10">
         <v>9.9130000000000003</v>
       </c>
-    </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O61" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P61" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" s="13">
         <v>30</v>
       </c>
@@ -3234,8 +3703,14 @@
       <c r="N62" s="10">
         <v>35.936</v>
       </c>
-    </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O62" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P62" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" s="3">
         <v>30</v>
       </c>
@@ -3278,8 +3753,14 @@
       <c r="N63" s="10">
         <v>6.782</v>
       </c>
-    </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O63" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P63" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" s="13">
         <v>30</v>
       </c>
@@ -3322,8 +3803,14 @@
       <c r="N64" s="10">
         <v>6.0839999999999996</v>
       </c>
-    </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O64" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P64" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" s="3">
         <v>30</v>
       </c>
@@ -3366,8 +3853,14 @@
       <c r="N65" s="10">
         <v>16.704000000000001</v>
       </c>
-    </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O65" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P65" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" s="13">
         <v>30</v>
       </c>
@@ -3410,8 +3903,14 @@
       <c r="N66" s="10">
         <v>12.16</v>
       </c>
-    </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O66" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P66" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" s="3">
         <v>30</v>
       </c>
@@ -3454,8 +3953,14 @@
       <c r="N67" s="10">
         <v>10.1</v>
       </c>
-    </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O67" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P67" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" s="13">
         <v>30</v>
       </c>
@@ -3498,8 +4003,14 @@
       <c r="N68" s="10">
         <v>7.9660000000000002</v>
       </c>
-    </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O68" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P68" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
         <v>30</v>
       </c>
@@ -3542,8 +4053,14 @@
       <c r="N69" s="10">
         <v>20.091000000000001</v>
       </c>
-    </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O69" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P69" s="18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" s="13">
         <v>30</v>
       </c>
@@ -3586,8 +4103,14 @@
       <c r="N70" s="10">
         <v>19.337</v>
       </c>
-    </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O70" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P70" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71" s="3">
         <v>30</v>
       </c>
@@ -3630,8 +4153,14 @@
       <c r="N71" s="10">
         <v>17.690000000000001</v>
       </c>
-    </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O71" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P71" s="18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" s="13">
         <v>30</v>
       </c>
@@ -3674,8 +4203,14 @@
       <c r="N72" s="10">
         <v>21.367999999999999</v>
       </c>
-    </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O72" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P72" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73" s="3">
         <v>30</v>
       </c>
@@ -3718,8 +4253,14 @@
       <c r="N73" s="10">
         <v>21.100999999999999</v>
       </c>
-    </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O73" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P73" s="18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74" s="13">
         <v>30</v>
       </c>
@@ -3762,8 +4303,14 @@
       <c r="N74" s="10">
         <v>25.388000000000002</v>
       </c>
-    </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O74" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P74" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" s="3">
         <v>30</v>
       </c>
@@ -3806,8 +4353,14 @@
       <c r="N75" s="10">
         <v>20.407</v>
       </c>
-    </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O75" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P75" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" s="13">
         <v>30</v>
       </c>
@@ -3850,8 +4403,14 @@
       <c r="N76" s="10">
         <v>20.036000000000001</v>
       </c>
-    </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O76" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P76" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" s="3">
         <v>30</v>
       </c>
@@ -3894,8 +4453,14 @@
       <c r="N77" s="10">
         <v>28.696000000000002</v>
       </c>
-    </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O77" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P77" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78" s="13">
         <v>30</v>
       </c>
@@ -3938,8 +4503,14 @@
       <c r="N78" s="10">
         <v>51.96</v>
       </c>
-    </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O78" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P78" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79" s="3">
         <v>30</v>
       </c>
@@ -3982,8 +4553,14 @@
       <c r="N79" s="10">
         <v>60.281999999999996</v>
       </c>
-    </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O79" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P79" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80" s="13">
         <v>30</v>
       </c>
@@ -4026,8 +4603,14 @@
       <c r="N80" s="10">
         <v>42.662999999999997</v>
       </c>
-    </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O80" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P80" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A81" s="3">
         <v>42</v>
       </c>
@@ -4070,8 +4653,14 @@
       <c r="N81" s="10">
         <v>0.60199999999999998</v>
       </c>
-    </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O81" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P81" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A82" s="13">
         <v>42</v>
       </c>
@@ -4114,8 +4703,14 @@
       <c r="N82" s="10">
         <v>3.4510000000000001</v>
       </c>
-    </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O82" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P82" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A83" s="3">
         <v>42</v>
       </c>
@@ -4158,8 +4753,14 @@
       <c r="N83" s="10">
         <v>1.5640000000000001</v>
       </c>
-    </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O83" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P83" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A84" s="13">
         <v>42</v>
       </c>
@@ -4202,8 +4803,14 @@
       <c r="N84" s="10">
         <v>1.355</v>
       </c>
-    </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O84" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P84" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A85" s="3">
         <v>42</v>
       </c>
@@ -4246,8 +4853,14 @@
       <c r="N85" s="10">
         <v>1.349</v>
       </c>
-    </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O85" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P85" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A86" s="13">
         <v>42</v>
       </c>
@@ -4290,8 +4903,14 @@
       <c r="N86" s="10">
         <v>3.8780000000000001</v>
       </c>
-    </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O86" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P86" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A87" s="3">
         <v>42</v>
       </c>
@@ -4334,8 +4953,14 @@
       <c r="N87" s="10">
         <v>8.9629999999999992</v>
       </c>
-    </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O87" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="P87" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A88" s="13">
         <v>42</v>
       </c>
@@ -4378,8 +5003,14 @@
       <c r="N88" s="10">
         <v>1.077</v>
       </c>
-    </row>
-    <row r="89" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O88" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P88" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A89" s="3">
         <v>42</v>
       </c>
@@ -4422,8 +5053,14 @@
       <c r="N89" s="10">
         <v>6.4539999999999997</v>
       </c>
-    </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O89" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P89" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A90" s="13">
         <v>42</v>
       </c>
@@ -4466,8 +5103,14 @@
       <c r="N90" s="10">
         <v>8.9440000000000008</v>
       </c>
-    </row>
-    <row r="91" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O90" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P90" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A91" s="3">
         <v>42</v>
       </c>
@@ -4510,8 +5153,14 @@
       <c r="N91" s="10">
         <v>4.0259999999999998</v>
       </c>
-    </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O91" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P91" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A92" s="13">
         <v>42</v>
       </c>
@@ -4554,8 +5203,14 @@
       <c r="N92" s="10">
         <v>7.2750000000000004</v>
       </c>
-    </row>
-    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O92" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P92" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A93" s="3">
         <v>42</v>
       </c>
@@ -4598,8 +5253,14 @@
       <c r="N93" s="10">
         <v>13.920999999999999</v>
       </c>
-    </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O93" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P93" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A94" s="13">
         <v>42</v>
       </c>
@@ -4642,8 +5303,14 @@
       <c r="N94" s="10">
         <v>8.1620000000000008</v>
       </c>
-    </row>
-    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O94" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P94" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A95" s="3">
         <v>42</v>
       </c>
@@ -4686,8 +5353,14 @@
       <c r="N95" s="10">
         <v>6.1929999999999996</v>
       </c>
-    </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O95" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P95" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A96" s="13">
         <v>42</v>
       </c>
@@ -4730,8 +5403,14 @@
       <c r="N96" s="10">
         <v>3.7330000000000001</v>
       </c>
-    </row>
-    <row r="97" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O96" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P96" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="97" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A97" s="3">
         <v>42</v>
       </c>
@@ -4774,8 +5453,14 @@
       <c r="N97" s="10">
         <v>32.198999999999998</v>
       </c>
-    </row>
-    <row r="98" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O97" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P97" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="98" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A98" s="13">
         <v>42</v>
       </c>
@@ -4818,8 +5503,14 @@
       <c r="N98" s="10">
         <v>13.926</v>
       </c>
-    </row>
-    <row r="99" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O98" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P98" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="99" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A99" s="3">
         <v>42</v>
       </c>
@@ -4862,8 +5553,14 @@
       <c r="N99" s="10">
         <v>6.2709999999999999</v>
       </c>
-    </row>
-    <row r="100" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O99" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P99" s="18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="100" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A100" s="13">
         <v>42</v>
       </c>
@@ -4906,8 +5603,14 @@
       <c r="N100" s="10">
         <v>11.632999999999999</v>
       </c>
-    </row>
-    <row r="101" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O100" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P100" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="101" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A101" s="3">
         <v>42</v>
       </c>
@@ -4950,8 +5653,14 @@
       <c r="N101" s="10">
         <v>25.114999999999998</v>
       </c>
-    </row>
-    <row r="102" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O101" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P101" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="102" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A102" s="13">
         <v>42</v>
       </c>
@@ -4994,8 +5703,14 @@
       <c r="N102" s="10">
         <v>12.106</v>
       </c>
-    </row>
-    <row r="103" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O102" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P102" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="103" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A103" s="3">
         <v>42</v>
       </c>
@@ -5038,8 +5753,14 @@
       <c r="N103" s="10">
         <v>20.631</v>
       </c>
-    </row>
-    <row r="104" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O103" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P103" s="18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="104" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A104" s="13">
         <v>42</v>
       </c>
@@ -5082,8 +5803,14 @@
       <c r="N104" s="10">
         <v>13.443</v>
       </c>
-    </row>
-    <row r="105" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O104" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P104" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="105" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A105" s="3">
         <v>42</v>
       </c>
@@ -5126,8 +5853,14 @@
       <c r="N105" s="10">
         <v>19.658999999999999</v>
       </c>
-    </row>
-    <row r="106" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O105" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P105" s="18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="106" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A106" s="13">
         <v>42</v>
       </c>
@@ -5170,8 +5903,14 @@
       <c r="N106" s="10">
         <v>16.623999999999999</v>
       </c>
-    </row>
-    <row r="107" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O106" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P106" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="107" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A107" s="3">
         <v>42</v>
       </c>
@@ -5214,8 +5953,14 @@
       <c r="N107" s="10">
         <v>17.387</v>
       </c>
-    </row>
-    <row r="108" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O107" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P107" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="108" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A108" s="13">
         <v>42</v>
       </c>
@@ -5258,8 +6003,14 @@
       <c r="N108" s="10">
         <v>25.341999999999999</v>
       </c>
-    </row>
-    <row r="109" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O108" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P108" s="18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="109" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A109" s="3">
         <v>42</v>
       </c>
@@ -5302,8 +6053,14 @@
       <c r="N109" s="10">
         <v>34.305</v>
       </c>
-    </row>
-    <row r="110" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O109" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P109" s="18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="110" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A110" s="13">
         <v>42</v>
       </c>
@@ -5346,8 +6103,14 @@
       <c r="N110" s="10">
         <v>30.234000000000002</v>
       </c>
-    </row>
-    <row r="111" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O110" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P110" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="111" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A111" s="3">
         <v>42</v>
       </c>
@@ -5390,8 +6153,14 @@
       <c r="N111" s="10">
         <v>22.872</v>
       </c>
-    </row>
-    <row r="112" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O111" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P111" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="112" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A112" s="13">
         <v>42</v>
       </c>
@@ -5434,8 +6203,14 @@
       <c r="N112" s="10">
         <v>32.244</v>
       </c>
-    </row>
-    <row r="113" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O112" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P112" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="113" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A113" s="3">
         <v>42</v>
       </c>
@@ -5478,8 +6253,14 @@
       <c r="N113" s="10">
         <v>60.542999999999999</v>
       </c>
-    </row>
-    <row r="114" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O113" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P113" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="114" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A114" s="13">
         <v>42</v>
       </c>
@@ -5522,8 +6303,14 @@
       <c r="N114" s="10">
         <v>72.605999999999995</v>
       </c>
-    </row>
-    <row r="115" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O114" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P114" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="115" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A115" s="3">
         <v>42</v>
       </c>
@@ -5566,8 +6353,14 @@
       <c r="N115" s="10">
         <v>191.155</v>
       </c>
-    </row>
-    <row r="116" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O115" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P115" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="116" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A116" s="13">
         <v>42</v>
       </c>
@@ -5610,13 +6403,20 @@
       <c r="N116" s="10">
         <v>64.266000000000005</v>
       </c>
+      <c r="O116" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P116" s="16" t="s">
+        <v>14</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
     <mergeCell ref="M1:N1"/>
-    <mergeCell ref="K1:L1"/>
     <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5625,7 +6425,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:N60"/>
+  <dimension ref="A1:P60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="6" customWidth="1"/>
@@ -5638,80 +6438,91 @@
     <col min="11" max="11" width="12" customWidth="1"/>
     <col min="12" max="12" width="10" customWidth="1"/>
     <col min="13" max="13" width="12" customWidth="1"/>
-    <col min="14" max="14" width="10" customWidth="1"/>
+    <col min="14" max="15" width="10" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="16"/>
-      <c r="I1" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="J1" s="16"/>
-      <c r="K1" s="15" t="s">
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="20"/>
+      <c r="I1" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="J1" s="20"/>
+      <c r="K1" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="L1" s="20"/>
+      <c r="M1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="L1" s="16"/>
-      <c r="M1" s="15" t="s">
+      <c r="N1" s="20"/>
+      <c r="O1" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="P1" s="23"/>
+    </row>
+    <row r="2" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="O2" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="N1" s="16"/>
-    </row>
-    <row r="2" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="P2" s="15" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>10</v>
       </c>
@@ -5754,8 +6565,14 @@
       <c r="N3" s="10">
         <v>0.999</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O3" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P3" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="13">
         <v>10</v>
       </c>
@@ -5798,8 +6615,14 @@
       <c r="N4" s="10">
         <v>1.5069999999999999</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O4" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P4" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>10</v>
       </c>
@@ -5842,8 +6665,14 @@
       <c r="N5" s="10">
         <v>0.64100000000000001</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O5" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P5" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="13">
         <v>10</v>
       </c>
@@ -5886,8 +6715,14 @@
       <c r="N6" s="10">
         <v>5.1970000000000001</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O6" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P6" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>10</v>
       </c>
@@ -5930,8 +6765,14 @@
       <c r="N7" s="10">
         <v>1.56</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O7" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P7" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="13">
         <v>10</v>
       </c>
@@ -5974,8 +6815,14 @@
       <c r="N8" s="10">
         <v>0.83899999999999997</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O8" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P8" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>10</v>
       </c>
@@ -6018,8 +6865,14 @@
       <c r="N9" s="10">
         <v>3.9409999999999998</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O9" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P9" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="13">
         <v>10</v>
       </c>
@@ -6062,8 +6915,14 @@
       <c r="N10" s="10">
         <v>2.6850000000000001</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O10" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P10" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -6106,8 +6965,14 @@
       <c r="N11" s="10">
         <v>2.2959999999999998</v>
       </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O11" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P11" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="13">
         <v>10</v>
       </c>
@@ -6150,8 +7015,14 @@
       <c r="N12" s="10">
         <v>9.5649999999999995</v>
       </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O12" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P12" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>25</v>
       </c>
@@ -6194,8 +7065,14 @@
       <c r="N13" s="10">
         <v>1.274</v>
       </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O13" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P13" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="13">
         <v>25</v>
       </c>
@@ -6238,8 +7115,14 @@
       <c r="N14" s="10">
         <v>3.4350000000000001</v>
       </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O14" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P14" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>25</v>
       </c>
@@ -6282,8 +7165,14 @@
       <c r="N15" s="10">
         <v>4.3079999999999998</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O15" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P15" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="13">
         <v>25</v>
       </c>
@@ -6326,8 +7215,14 @@
       <c r="N16" s="10">
         <v>1.7030000000000001</v>
       </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O16" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P16" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>25</v>
       </c>
@@ -6370,8 +7265,14 @@
       <c r="N17" s="10">
         <v>9.702</v>
       </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O17" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P17" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="13">
         <v>25</v>
       </c>
@@ -6414,8 +7315,14 @@
       <c r="N18" s="10">
         <v>6.1870000000000003</v>
       </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O18" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P18" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>25</v>
       </c>
@@ -6458,8 +7365,14 @@
       <c r="N19" s="10">
         <v>6.6319999999999997</v>
       </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O19" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P19" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="13">
         <v>25</v>
       </c>
@@ -6502,8 +7415,14 @@
       <c r="N20" s="10">
         <v>31.434000000000001</v>
       </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O20" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="P20" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>25</v>
       </c>
@@ -6546,8 +7465,14 @@
       <c r="N21" s="10">
         <v>13.948</v>
       </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O21" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P21" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="13">
         <v>25</v>
       </c>
@@ -6590,8 +7515,14 @@
       <c r="N22" s="10">
         <v>8.18</v>
       </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O22" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P22" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>25</v>
       </c>
@@ -6634,8 +7565,14 @@
       <c r="N23" s="10">
         <v>15.186</v>
       </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O23" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P23" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="13">
         <v>25</v>
       </c>
@@ -6678,8 +7615,14 @@
       <c r="N24" s="10">
         <v>37.573999999999998</v>
       </c>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O24" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P24" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>25</v>
       </c>
@@ -6722,8 +7665,14 @@
       <c r="N25" s="10">
         <v>12.122</v>
       </c>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O25" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P25" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="13">
         <v>25</v>
       </c>
@@ -6766,8 +7715,14 @@
       <c r="N26" s="10">
         <v>37.512999999999998</v>
       </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O26" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P26" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>25</v>
       </c>
@@ -6810,8 +7765,14 @@
       <c r="N27" s="10">
         <v>25.396000000000001</v>
       </c>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O27" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P27" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="13">
         <v>25</v>
       </c>
@@ -6854,8 +7815,14 @@
       <c r="N28" s="10">
         <v>24.885999999999999</v>
       </c>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O28" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P28" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>25</v>
       </c>
@@ -6898,8 +7865,14 @@
       <c r="N29" s="10">
         <v>26.509</v>
       </c>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O29" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="P29" s="18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="13">
         <v>25</v>
       </c>
@@ -6942,8 +7915,14 @@
       <c r="N30" s="10">
         <v>42.170999999999999</v>
       </c>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O30" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P30" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -6986,8 +7965,14 @@
       <c r="N31" s="10">
         <v>4.1120000000000001</v>
       </c>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O31" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P31" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="13">
         <v>30</v>
       </c>
@@ -7030,8 +8015,14 @@
       <c r="N32" s="10">
         <v>4.2469999999999999</v>
       </c>
-    </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O32" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P32" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>30</v>
       </c>
@@ -7074,8 +8065,14 @@
       <c r="N33" s="10">
         <v>3.2869999999999999</v>
       </c>
-    </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O33" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P33" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" s="13">
         <v>30</v>
       </c>
@@ -7118,8 +8115,14 @@
       <c r="N34" s="10">
         <v>17.102</v>
       </c>
-    </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O34" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P34" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>30</v>
       </c>
@@ -7162,8 +8165,14 @@
       <c r="N35" s="10">
         <v>15.597</v>
       </c>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O35" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P35" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="13">
         <v>30</v>
       </c>
@@ -7206,8 +8215,14 @@
       <c r="N36" s="10">
         <v>3.532</v>
       </c>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O36" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P36" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>30</v>
       </c>
@@ -7250,8 +8265,14 @@
       <c r="N37" s="10">
         <v>8.6549999999999994</v>
       </c>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O37" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="P37" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" s="13">
         <v>30</v>
       </c>
@@ -7294,8 +8315,14 @@
       <c r="N38" s="10">
         <v>10.247</v>
       </c>
-    </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O38" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P38" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>30</v>
       </c>
@@ -7338,8 +8365,14 @@
       <c r="N39" s="10">
         <v>6.1520000000000001</v>
       </c>
-    </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O39" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P39" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="13">
         <v>30</v>
       </c>
@@ -7382,8 +8415,14 @@
       <c r="N40" s="10">
         <v>13.864000000000001</v>
       </c>
-    </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O40" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="P40" s="18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>30</v>
       </c>
@@ -7426,8 +8465,14 @@
       <c r="N41" s="10">
         <v>9.8979999999999997</v>
       </c>
-    </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O41" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P41" s="18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" s="13">
         <v>30</v>
       </c>
@@ -7470,8 +8515,14 @@
       <c r="N42" s="10">
         <v>18.358000000000001</v>
       </c>
-    </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O42" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P42" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>30</v>
       </c>
@@ -7514,8 +8565,14 @@
       <c r="N43" s="10">
         <v>51.93</v>
       </c>
-    </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O43" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="P43" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" s="13">
         <v>30</v>
       </c>
@@ -7558,8 +8615,14 @@
       <c r="N44" s="10">
         <v>42.469000000000001</v>
       </c>
-    </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O44" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P44" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>30</v>
       </c>
@@ -7602,8 +8665,14 @@
       <c r="N45" s="10">
         <v>25.143999999999998</v>
       </c>
-    </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O45" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P45" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="13">
         <v>42</v>
       </c>
@@ -7646,8 +8715,14 @@
       <c r="N46" s="10">
         <v>2.9289999999999998</v>
       </c>
-    </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O46" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P46" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>42</v>
       </c>
@@ -7690,8 +8765,14 @@
       <c r="N47" s="10">
         <v>8.2859999999999996</v>
       </c>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O47" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="P47" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" s="13">
         <v>42</v>
       </c>
@@ -7734,8 +8815,14 @@
       <c r="N48" s="10">
         <v>5.42</v>
       </c>
-    </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O48" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P48" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>42</v>
       </c>
@@ -7778,8 +8865,14 @@
       <c r="N49" s="10">
         <v>8.1929999999999996</v>
       </c>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O49" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P49" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="13">
         <v>42</v>
       </c>
@@ -7822,8 +8915,14 @@
       <c r="N50" s="10">
         <v>6.891</v>
       </c>
-    </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O50" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P50" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <v>42</v>
       </c>
@@ -7866,8 +8965,14 @@
       <c r="N51" s="10">
         <v>6.7439999999999998</v>
       </c>
-    </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O51" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P51" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" s="13">
         <v>42</v>
       </c>
@@ -7910,8 +9015,14 @@
       <c r="N52" s="10">
         <v>11.013</v>
       </c>
-    </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O52" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="P52" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>42</v>
       </c>
@@ -7954,8 +9065,14 @@
       <c r="N53" s="10">
         <v>9.7899999999999991</v>
       </c>
-    </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O53" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="P53" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="13">
         <v>42</v>
       </c>
@@ -7998,8 +9115,14 @@
       <c r="N54" s="10">
         <v>22.047000000000001</v>
       </c>
-    </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O54" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P54" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>42</v>
       </c>
@@ -8042,8 +9165,14 @@
       <c r="N55" s="10">
         <v>38.094999999999999</v>
       </c>
-    </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O55" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P55" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" s="13">
         <v>42</v>
       </c>
@@ -8086,8 +9215,14 @@
       <c r="N56" s="10">
         <v>15.727</v>
       </c>
-    </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O56" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="P56" s="18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>42</v>
       </c>
@@ -8130,8 +9265,14 @@
       <c r="N57" s="10">
         <v>49.978000000000002</v>
       </c>
-    </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O57" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="P57" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" s="13">
         <v>42</v>
       </c>
@@ -8174,8 +9315,14 @@
       <c r="N58" s="10">
         <v>57.03</v>
       </c>
-    </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O58" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="P58" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>42</v>
       </c>
@@ -8218,8 +9365,14 @@
       <c r="N59" s="10">
         <v>199.08199999999999</v>
       </c>
-    </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O59" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="P59" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" s="13">
         <v>42</v>
       </c>
@@ -8262,13 +9415,20 @@
       <c r="N60" s="10">
         <v>71.113</v>
       </c>
+      <c r="O60" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="P60" s="17" t="s">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="O1:P1"/>
     <mergeCell ref="M1:N1"/>
-    <mergeCell ref="K1:L1"/>
     <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>